<commit_message>
feat: Story 0.5 calc-service scaffold + CI/CD pipeline + infra updates (Stories 0.5 & 0.6)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bmad/_bmad-output/planning-artifacts/cost-tracker/Star-Energy-CEMS-Cost-Tracker.xlsx
+++ b/docs/bmad/_bmad-output/planning-artifacts/cost-tracker/Star-Energy-CEMS-Cost-Tracker.xlsx
@@ -1372,7 +1372,9 @@
         <f>E4*F4</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="n"/>
+      <c r="H4" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="I4" s="14">
         <f>H4*F4</f>
         <v/>
@@ -1427,7 +1429,9 @@
         <f>E5*F5</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="n"/>
+      <c r="H5" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" s="14">
         <f>H5*F5</f>
         <v/>
@@ -1482,7 +1486,9 @@
         <f>E6*F6</f>
         <v/>
       </c>
-      <c r="H6" s="7" t="n"/>
+      <c r="H6" s="7" t="n">
+        <v>12</v>
+      </c>
       <c r="I6" s="14">
         <f>H6*F6</f>
         <v/>
@@ -1497,7 +1503,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>in-progress</t>
+          <t>done</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
@@ -1537,7 +1543,9 @@
         <f>E7*F7</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="n"/>
+      <c r="H7" s="7" t="n">
+        <v>12</v>
+      </c>
       <c r="I7" s="14">
         <f>H7*F7</f>
         <v/>
@@ -1552,63 +1560,69 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>backlog</t>
-        </is>
-      </c>
-      <c r="M7" s="6" t="inlineStr"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>Completed 2026-04-28</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Epic 0</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>0-5</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Python calculation service scaffold</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="E8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="28" t="n">
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="G8" s="29">
+      <c r="G8" s="14">
         <f>E8*F8</f>
         <v/>
       </c>
-      <c r="H8" s="27" t="n"/>
-      <c r="I8" s="29">
+      <c r="H8" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="I8" s="14">
         <f>H8*F8</f>
         <v/>
       </c>
-      <c r="J8" s="27">
+      <c r="J8" s="7">
         <f>H8-E8</f>
         <v/>
       </c>
-      <c r="K8" s="29">
+      <c r="K8" s="14">
         <f>I8-G8</f>
         <v/>
       </c>
-      <c r="L8" s="26" t="inlineStr">
-        <is>
-          <t>deferred</t>
-        </is>
-      </c>
-      <c r="M8" s="26" t="inlineStr">
-        <is>
-          <t>Consolidate calcs into Node for MVP</t>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>Built despite deferral — needed for CI/CD integration (2026-04-28)</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1657,9 @@
         <f>E9*F9</f>
         <v/>
       </c>
-      <c r="H9" s="7" t="n"/>
+      <c r="H9" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="I9" s="14">
         <f>H9*F9</f>
         <v/>
@@ -1658,12 +1674,12 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>done</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>Basic GitHub Actions</t>
+          <t>Completed 2026-05-01; complex OIDC + slot-swap wiring</t>
         </is>
       </c>
     </row>
@@ -8243,7 +8259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8430,180 +8446,248 @@
       <c r="F7" s="48" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Story execution</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Story 0-3 DB schema + RLS — completed (12 hrs est)</t>
+        </is>
+      </c>
+      <c r="F8" s="48" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Story execution</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Story 0-4 Node.js API foundation + BullMQ — completed (12 hrs est)</t>
+        </is>
+      </c>
+      <c r="F9" s="48" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Story execution</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Story 0-5 Python calc service scaffold — completed despite deferral (8 hrs est)</t>
+        </is>
+      </c>
+      <c r="F10" s="48" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Story execution</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Story 0-6 CI/CD pipeline + OIDC/slot-swap — completed (10 hrs actual vs 6 est)</t>
+        </is>
+      </c>
+      <c r="F11" s="48" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
           <t>Subscriptions</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Claude Max 20x</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Anthropic</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Monthly subscription</t>
-        </is>
-      </c>
-      <c r="F8" s="48" t="n">
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>April subscription cycle</t>
+        </is>
+      </c>
+      <c r="F12" s="48" t="n">
         <v>200</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Subscriptions</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>GitHub Free</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>GitHub</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>No charge</t>
         </is>
       </c>
-      <c r="F9" s="48" t="n">
+      <c r="F13" s="48" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Azure dev environment</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>First bill ~30 days after provisioning</t>
         </is>
       </c>
-      <c r="F10" s="48" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="F14" s="48" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>One-time</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>TBD registrar</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>starenergy-cems.com (or similar)</t>
         </is>
       </c>
-      <c r="F11" s="48" t="n">
+      <c r="F15" s="48" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>One-time</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Legal templates</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Termly</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>T&amp;Cs + Privacy</t>
         </is>
       </c>
-      <c r="F12" s="48" t="n">
+      <c r="F16" s="48" t="n">
         <v>50</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -8917,24 +9001,72 @@
       <c r="I42" s="5" t="n"/>
       <c r="J42" s="5" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="5" t="n"/>
+      <c r="B43" s="5" t="n"/>
+      <c r="C43" s="5" t="n"/>
+      <c r="D43" s="5" t="n"/>
+      <c r="E43" s="5" t="n"/>
+      <c r="F43" s="14" t="n"/>
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="5" t="n"/>
+      <c r="I43" s="5" t="n"/>
+      <c r="J43" s="5" t="n"/>
+    </row>
     <row r="44">
-      <c r="A44" s="35" t="n"/>
-      <c r="B44" s="35" t="n"/>
-      <c r="C44" s="35" t="n"/>
-      <c r="D44" s="35" t="n"/>
-      <c r="E44" s="35" t="inlineStr">
+      <c r="A44" s="5" t="n"/>
+      <c r="B44" s="5" t="n"/>
+      <c r="C44" s="5" t="n"/>
+      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="14" t="n"/>
+      <c r="G44" s="5" t="n"/>
+      <c r="H44" s="5" t="n"/>
+      <c r="I44" s="5" t="n"/>
+      <c r="J44" s="5" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n"/>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="14" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="5" t="n"/>
+      <c r="I45" s="5" t="n"/>
+      <c r="J45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n"/>
+      <c r="B46" s="5" t="n"/>
+      <c r="C46" s="5" t="n"/>
+      <c r="D46" s="5" t="n"/>
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="14" t="n"/>
+      <c r="G46" s="5" t="n"/>
+      <c r="H46" s="5" t="n"/>
+      <c r="I46" s="5" t="n"/>
+      <c r="J46" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="35" t="n"/>
+      <c r="B48" s="35" t="n"/>
+      <c r="C48" s="35" t="n"/>
+      <c r="D48" s="35" t="n"/>
+      <c r="E48" s="35" t="inlineStr">
         <is>
           <t>TOTAL ACTUAL SPEND (cash)</t>
         </is>
       </c>
-      <c r="F44" s="38">
-        <f>SUM(F4:F42)</f>
-        <v/>
-      </c>
-      <c r="G44" s="35" t="n"/>
-      <c r="H44" s="35" t="n"/>
-      <c r="I44" s="35" t="n"/>
-      <c r="J44" s="35" t="n"/>
+      <c r="F48" s="38">
+        <f>SUM(F4:F46)</f>
+        <v/>
+      </c>
+      <c r="G48" s="35" t="n"/>
+      <c r="H48" s="35" t="n"/>
+      <c r="I48" s="35" t="n"/>
+      <c r="J48" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>